<commit_message>
After Tech review (still need to re-update yr19 and yr20 GS CV files, which needed to use the updated individual measurements value)
</commit_message>
<xml_diff>
--- a/TraitAnalyses201003/data/Genetic_Cor_between_years.xlsx
+++ b/TraitAnalyses201003/data/Genetic_Cor_between_years.xlsx
@@ -4,12 +4,15 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="27729"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="620" yWindow="720" windowWidth="23920" windowHeight="13200" tabRatio="500"/>
+    <workbookView xWindow="1140" yWindow="0" windowWidth="23920" windowHeight="13260" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Genetic_cor_among_3YRs" sheetId="1" r:id="rId1"/>
+    <sheet name="Genetic_cor_among_3YRs_WRONG" sheetId="1" r:id="rId1"/>
     <sheet name="GBLUP_among_3YRs" sheetId="2" r:id="rId2"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
   <calcPr calcId="140000" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
@@ -20,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="30">
   <si>
     <t>Yr19_Yr20</t>
   </si>
@@ -67,42 +70,18 @@
     <t>GBLUP</t>
   </si>
   <si>
-    <t>Yr20_Yr19</t>
-  </si>
-  <si>
-    <t>WWP</t>
-  </si>
-  <si>
     <t>pDW</t>
   </si>
   <si>
     <t>DWpM</t>
   </si>
   <si>
-    <t>Ash</t>
-  </si>
-  <si>
-    <t>AshFDWpM</t>
-  </si>
-  <si>
-    <t>DP</t>
-  </si>
-  <si>
-    <t>Blen</t>
-  </si>
-  <si>
     <t>BmWid</t>
   </si>
   <si>
     <t>BTh</t>
   </si>
   <si>
-    <t>Slen</t>
-  </si>
-  <si>
-    <t>SDia</t>
-  </si>
-  <si>
     <t>wetWgtPlot</t>
   </si>
   <si>
@@ -110,13 +89,37 @@
   </si>
   <si>
     <t>h2</t>
+  </si>
+  <si>
+    <t>BL</t>
+  </si>
+  <si>
+    <t>SL</t>
+  </si>
+  <si>
+    <t>07172021 Corrected for indiv traits</t>
+  </si>
+  <si>
+    <t>WWpM</t>
+  </si>
+  <si>
+    <t>BD</t>
+  </si>
+  <si>
+    <t>Sdia</t>
+  </si>
+  <si>
+    <t>Yr19 predict Yr20</t>
+  </si>
+  <si>
+    <t>Yr20 predict Yr19</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -152,6 +155,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -183,7 +193,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="35">
+  <cellStyleXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -219,16 +229,52 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="35">
+  <cellStyles count="69">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -246,6 +292,23 @@
     <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="44" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="46" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="48" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="50" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="52" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="54" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="56" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="58" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="60" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="62" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="64" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="66" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="68" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -263,6 +326,23 @@
     <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="43" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="45" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="47" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="49" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="51" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="53" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="55" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="57" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="59" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="61" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="63" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="65" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="67" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -310,7 +390,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Genetic_cor_among_3YRs!$A$9:$A$16</c:f>
+              <c:f>Genetic_cor_among_3YRs_WRONG!$A$9:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -319,7 +399,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Genetic_cor_among_3YRs!$C$9:$C$16</c:f>
+              <c:f>Genetic_cor_among_3YRs_WRONG!$C$9:$C$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -360,7 +440,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Genetic_cor_among_3YRs!$A$9:$A$16</c:f>
+              <c:f>Genetic_cor_among_3YRs_WRONG!$A$9:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -369,7 +449,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Genetic_cor_among_3YRs!$D$9:$D$16</c:f>
+              <c:f>Genetic_cor_among_3YRs_WRONG!$D$9:$D$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -410,7 +490,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Genetic_cor_among_3YRs!$A$9:$A$16</c:f>
+              <c:f>Genetic_cor_among_3YRs_WRONG!$A$9:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -419,7 +499,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Genetic_cor_among_3YRs!$E$9:$E$16</c:f>
+              <c:f>Genetic_cor_among_3YRs_WRONG!$E$9:$E$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -530,7 +610,17 @@
   <c:chart>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.0674720999441999"/>
+          <c:y val="0.0769230769230769"/>
+          <c:w val="0.727834025668051"/>
+          <c:h val="0.67400399045142"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -543,71 +633,76 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="558ED5"/>
+              <a:schemeClr val="accent6">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
             </a:solidFill>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>GBLUP_among_3YRs!$B$24:$I$24</c:f>
+              <c:f>GBLUP_among_3YRs!$C$5:$K$5</c:f>
               <c:strCache>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>WWP</c:v>
+                  <c:v>DWpM</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>DWpM</c:v>
+                  <c:v>WWpM</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>DP</c:v>
+                  <c:v>pDW</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Blen</c:v>
+                  <c:v>BD</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>BL</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>BmWid</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>BTh</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>Slen</c:v>
-                </c:pt>
                 <c:pt idx="7">
-                  <c:v>SDia</c:v>
+                  <c:v>SL</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sdia</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>GBLUP_among_3YRs!$B$2:$I$2</c:f>
+              <c:f>GBLUP_among_3YRs!$C$2:$K$2</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.241151454801338</c:v>
+                  <c:v>0.21500835339038</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.197747787555113</c:v>
+                  <c:v>0.240378717428011</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.0173971939809785</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>-0.254486236263905</c:v>
+                  <c:v>0.0295925429399892</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-0.145458353777632</c:v>
+                  <c:v>0.239421408540162</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.0739909426248793</c:v>
+                  <c:v>0.303746788255227</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-0.154791795524483</c:v>
+                  <c:v>0.0783719816893105</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.512848587332577</c:v>
+                  <c:v>0.382979129536068</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.523695437375054</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -621,74 +716,79 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent6">
-                <a:lumMod val="60000"/>
-                <a:lumOff val="40000"/>
+              <a:schemeClr val="bg1">
+                <a:lumMod val="75000"/>
               </a:schemeClr>
             </a:solidFill>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>GBLUP_among_3YRs!$B$24:$I$24</c:f>
+              <c:f>GBLUP_among_3YRs!$C$5:$K$5</c:f>
               <c:strCache>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>WWP</c:v>
+                  <c:v>DWpM</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>DWpM</c:v>
+                  <c:v>WWpM</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>DP</c:v>
+                  <c:v>pDW</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Blen</c:v>
+                  <c:v>BD</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>BL</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>BmWid</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>BTh</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>Slen</c:v>
-                </c:pt>
                 <c:pt idx="7">
-                  <c:v>SDia</c:v>
+                  <c:v>SL</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sdia</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>GBLUP_among_3YRs!$B$3:$I$3</c:f>
+              <c:f>GBLUP_among_3YRs!$C$3:$K$3</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.286218469900732</c:v>
+                  <c:v>0.256987390249432</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.294112200299087</c:v>
+                  <c:v>0.025101560939601</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.2124078359963</c:v>
+                  <c:v>0.292892910691637</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0.273761633249357</c:v>
+                  <c:v>0.136077862251334</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-0.13717831006504</c:v>
+                  <c:v>0.370431795957093</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.0707064791594922</c:v>
+                  <c:v>0.388816944616789</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-0.0185399655390095</c:v>
+                  <c:v>0.0158280799174274</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.271926948825554</c:v>
+                  <c:v>0.26754431886759</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.240246883035268</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -700,68 +800,78 @@
           <c:tx>
             <c:v>TP: Yr2019+2020</c:v>
           </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>GBLUP_among_3YRs!$B$24:$I$24</c:f>
+              <c:f>GBLUP_among_3YRs!$C$5:$K$5</c:f>
               <c:strCache>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>WWP</c:v>
+                  <c:v>DWpM</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>DWpM</c:v>
+                  <c:v>WWpM</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>DP</c:v>
+                  <c:v>pDW</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Blen</c:v>
+                  <c:v>BD</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>BL</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>BmWid</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>BTh</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>Slen</c:v>
-                </c:pt>
                 <c:pt idx="7">
-                  <c:v>SDia</c:v>
+                  <c:v>SL</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sdia</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>GBLUP_among_3YRs!$B$4:$I$4</c:f>
+              <c:f>GBLUP_among_3YRs!$C$4:$K$4</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.294638002421637</c:v>
+                  <c:v>0.242671450704156</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.295359317493444</c:v>
+                  <c:v>0.0571035210275157</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.120496448136221</c:v>
+                  <c:v>0.227030305987779</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0.316067701819471</c:v>
+                  <c:v>0.0853063840243675</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-0.181660647595814</c:v>
+                  <c:v>0.164726082735345</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.0960455357533535</c:v>
+                  <c:v>0.319618423532567</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-0.0929601691862477</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.31892595579883</c:v>
+                  <c:v>0.0277352437125336</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.0641597402420307</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -790,6 +900,16 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
         <c:crossAx val="1959002760"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
@@ -804,7 +924,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -846,7 +966,17 @@
   <c:chart>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.0619905153901217"/>
+          <c:y val="0.0249480249480249"/>
+          <c:w val="0.841143521832498"/>
+          <c:h val="0.826986756593056"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -855,7 +985,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Yr19_Yr20</c:v>
+            <c:v>Yr19 predict Yr20</c:v>
           </c:tx>
           <c:spPr>
             <a:pattFill prst="ltDnDiag">
@@ -873,83 +1003,65 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>GBLUP_among_3YRs!$B$24:$L$24</c:f>
+              <c:f>GBLUP_among_3YRs!$C$5:$K$5</c:f>
               <c:strCache>
-                <c:ptCount val="11"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>WWP</c:v>
+                  <c:v>DWpM</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>DWpM</c:v>
+                  <c:v>WWpM</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>DP</c:v>
+                  <c:v>pDW</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Blen</c:v>
+                  <c:v>BD</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>BL</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>BmWid</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>BTh</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>Slen</c:v>
-                </c:pt>
                 <c:pt idx="7">
-                  <c:v>SDia</c:v>
+                  <c:v>SL</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>pDW</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Ash</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>AshFDWpM</c:v>
+                  <c:v>Sdia</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>GBLUP_among_3YRs!$B$25:$L$25</c:f>
+              <c:f>GBLUP_among_3YRs!$C$25:$K$25</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.193776965560342</c:v>
+                  <c:v>0.155014061</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.148640478110187</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>-0.0342117296386602</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.0773063172010051</c:v>
+                  <c:v>0.194315543</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.0747926931331445</c:v>
+                  <c:v>0.346087447</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.0447504928651784</c:v>
+                  <c:v>0.344955126</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.0704324800656173</c:v>
+                  <c:v>0.056733138</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.360484043101821</c:v>
+                  <c:v>0.325152607</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-0.0354047145057401</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>-0.0428184285195332</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>-0.0200433297450381</c:v>
+                  <c:v>0.360213727</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -959,7 +1071,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Yr20_Yr19</c:v>
+            <c:v>Yr20 predict Yr19</c:v>
           </c:tx>
           <c:spPr>
             <a:pattFill prst="ltDnDiag">
@@ -977,83 +1089,65 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>GBLUP_among_3YRs!$B$24:$L$24</c:f>
+              <c:f>GBLUP_among_3YRs!$C$5:$K$5</c:f>
               <c:strCache>
-                <c:ptCount val="11"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>WWP</c:v>
+                  <c:v>DWpM</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>DWpM</c:v>
+                  <c:v>WWpM</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>DP</c:v>
+                  <c:v>pDW</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Blen</c:v>
+                  <c:v>BD</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>BL</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>BmWid</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>BTh</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>Slen</c:v>
-                </c:pt>
                 <c:pt idx="7">
-                  <c:v>SDia</c:v>
+                  <c:v>SL</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>pDW</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Ash</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>AshFDWpM</c:v>
+                  <c:v>Sdia</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>GBLUP_among_3YRs!$B$26:$L$26</c:f>
+              <c:f>GBLUP_among_3YRs!$C$26:$K$26</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.279459754945589</c:v>
+                  <c:v>0.176212466433062</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.186479849778353</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>-0.0269432626058048</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.060648120765381</c:v>
+                  <c:v>0.242605311494363</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.194115642981616</c:v>
+                  <c:v>0.39478523849171</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.0397435614897588</c:v>
+                  <c:v>0.347969405722789</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.0110624733978087</c:v>
+                  <c:v>0.0624799965210711</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.450831557111153</c:v>
+                  <c:v>0.359808240288665</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-0.109231737842851</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>-0.0261391764377291</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>-0.01971692084842</c:v>
+                  <c:v>0.44984631182525</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1078,9 +1172,20 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
         <c:crossAx val="1964668712"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
@@ -1106,7 +1211,16 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.113671617752326"/>
+          <c:y val="0.0880128341545664"/>
+          <c:w val="0.203047423049392"/>
+          <c:h val="0.16700967472621"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -1160,16 +1274,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>368300</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>203200</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>69850</xdr:rowOff>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1191,15 +1305,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>196850</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1219,6 +1333,137 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Without_FMLoc_cor_BLUE_raw_mode"/>
+      <sheetName val="GS_cor_Table"/>
+      <sheetName val="Table1a_H2, 2a_GScor"/>
+      <sheetName val="Table1b_Gen_cor"/>
+      <sheetName val="Table 2b_BetweenLoc"/>
+      <sheetName val="GCA_SCA_varcomp95%"/>
+      <sheetName val="Mixed_PloidyT1a,2a,2b GCA95%"/>
+      <sheetName val="CompareModels_PlotLevelTraits_R"/>
+      <sheetName val="Mixed_Ploidy_T1a,2a,2b_950Indiv"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8">
+        <row r="1">
+          <cell r="C1" t="str">
+            <v>DWpM</v>
+          </cell>
+          <cell r="D1" t="str">
+            <v>WWpM</v>
+          </cell>
+          <cell r="E1" t="str">
+            <v>pDW</v>
+          </cell>
+          <cell r="F1" t="str">
+            <v>BD</v>
+          </cell>
+          <cell r="G1" t="str">
+            <v>BL</v>
+          </cell>
+          <cell r="H1" t="str">
+            <v>BmWid</v>
+          </cell>
+          <cell r="I1" t="str">
+            <v>BTh</v>
+          </cell>
+          <cell r="J1" t="str">
+            <v>SL</v>
+          </cell>
+          <cell r="K1" t="str">
+            <v>SDia</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="D15">
+            <v>0.88945351205616896</v>
+          </cell>
+          <cell r="E15">
+            <v>0.615620756341132</v>
+          </cell>
+          <cell r="G15">
+            <v>0.96093156709613403</v>
+          </cell>
+          <cell r="H15">
+            <v>0.80163384942932003</v>
+          </cell>
+          <cell r="I15">
+            <v>0.72588042095767402</v>
+          </cell>
+          <cell r="J15">
+            <v>0.60010286536858104</v>
+          </cell>
+          <cell r="K15">
+            <v>0.96775367476059704</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="C16">
+            <v>0.976087927904849</v>
+          </cell>
+          <cell r="D16">
+            <v>0.94633085022473395</v>
+          </cell>
+          <cell r="E16">
+            <v>0.94131140883727205</v>
+          </cell>
+          <cell r="F16">
+            <v>0.99468769043412097</v>
+          </cell>
+          <cell r="G16">
+            <v>0.93976448440246596</v>
+          </cell>
+          <cell r="H16">
+            <v>0.99677285358287504</v>
+          </cell>
+          <cell r="I16">
+            <v>0.89394449119885999</v>
+          </cell>
+          <cell r="J16">
+            <v>0.62392404651533595</v>
+          </cell>
+          <cell r="K16">
+            <v>0.73139892775372795</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="C17">
+            <v>0.52447135342901297</v>
+          </cell>
+          <cell r="D17">
+            <v>0.66961018354327895</v>
+          </cell>
+          <cell r="G17">
+            <v>0.57150566458222896</v>
+          </cell>
+          <cell r="H17">
+            <v>0.97282644459180101</v>
+          </cell>
+          <cell r="J17">
+            <v>0.70450645914651</v>
+          </cell>
+          <cell r="K17">
+            <v>0.96652710312355405</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1694,7 +1939,7 @@
         <v>2</v>
       </c>
       <c r="G8" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1731,7 +1976,7 @@
         <v>0.96037178045965998</v>
       </c>
       <c r="F10" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G10" s="2">
         <v>0.22758949807811901</v>
@@ -1751,7 +1996,7 @@
         <v>0.89655656366027103</v>
       </c>
       <c r="F11" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G11" s="2">
         <v>0.20348216371366301</v>
@@ -1893,238 +2138,289 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" t="s">
+    <row r="1" spans="1:13">
+      <c r="B1" t="s">
         <v>14</v>
-      </c>
-      <c r="B1" t="s">
-        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>6</v>
       </c>
       <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2">
-        <v>0.24115145480133801</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0.19774778755511299</v>
-      </c>
-      <c r="D2" s="2">
-        <v>1.7397193980978502E-2</v>
-      </c>
-      <c r="E2" s="2">
-        <v>-0.25448623626390499</v>
-      </c>
-      <c r="F2" s="2">
-        <v>-0.145458353777632</v>
-      </c>
-      <c r="G2" s="2">
-        <v>7.3990942624879305E-2</v>
-      </c>
-      <c r="H2" s="2">
-        <v>-0.15479179552448299</v>
-      </c>
-      <c r="I2" s="2">
-        <v>0.51284858733257699</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" t="s">
+      <c r="C2">
+        <v>0.21500835339037999</v>
+      </c>
+      <c r="D2">
+        <v>0.24037871742801101</v>
+      </c>
+      <c r="E2">
+        <v>2.9592542939989201E-2</v>
+      </c>
+      <c r="G2">
+        <v>0.239421408540162</v>
+      </c>
+      <c r="H2">
+        <v>0.303746788255227</v>
+      </c>
+      <c r="I2">
+        <v>7.8371981689310505E-2</v>
+      </c>
+      <c r="J2">
+        <v>0.382979129536068</v>
+      </c>
+      <c r="K2">
+        <v>0.52369543737505397</v>
+      </c>
+      <c r="M2">
+        <f>AVERAGE(C2:K4,F6,J6)</f>
+        <v>0.18869482545019328</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="B3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2">
-        <v>0.28621846990073202</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.29411220029908702</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.2124078359963</v>
-      </c>
-      <c r="E3" s="2">
-        <v>-0.27376163324935698</v>
-      </c>
-      <c r="F3" s="2">
-        <v>-0.13717831006504</v>
-      </c>
-      <c r="G3" s="2">
-        <v>7.07064791594922E-2</v>
-      </c>
-      <c r="H3" s="2">
-        <v>-1.8539965539009499E-2</v>
-      </c>
-      <c r="I3" s="2">
-        <v>0.27192694882555402</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" t="s">
+      <c r="C3">
+        <v>0.25698739024943201</v>
+      </c>
+      <c r="D3">
+        <v>2.5101560939601E-2</v>
+      </c>
+      <c r="E3">
+        <v>0.29289291069163698</v>
+      </c>
+      <c r="F3">
+        <v>0.136077862251334</v>
+      </c>
+      <c r="G3">
+        <v>0.37043179595709302</v>
+      </c>
+      <c r="H3">
+        <v>0.38881694461678901</v>
+      </c>
+      <c r="I3">
+        <v>1.58280799174274E-2</v>
+      </c>
+      <c r="J3">
+        <v>0.26754431886759</v>
+      </c>
+      <c r="K3">
+        <v>0.24024688303526801</v>
+      </c>
+      <c r="M3">
+        <f>AVERAGE(C2:K4)</f>
+        <v>0.20781893030586673</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="B4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="2">
-        <v>0.29463800242163701</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.29535931749344402</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.120496448136221</v>
-      </c>
-      <c r="E4" s="2">
-        <v>-0.31606770181947103</v>
-      </c>
-      <c r="F4" s="2">
-        <v>-0.18166064759581399</v>
-      </c>
-      <c r="G4" s="2">
-        <v>9.6045535753353506E-2</v>
-      </c>
-      <c r="H4" s="2">
-        <v>-9.2960169186247693E-2</v>
-      </c>
-      <c r="I4" s="2">
-        <v>0.31892595579882999</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" ht="16" thickBot="1"/>
-    <row r="24" spans="1:12" ht="16" thickBot="1">
-      <c r="A24" t="s">
+      <c r="C4">
+        <v>0.24267145070415599</v>
+      </c>
+      <c r="D4">
+        <v>5.7103521027515702E-2</v>
+      </c>
+      <c r="E4">
+        <v>0.22703030598777901</v>
+      </c>
+      <c r="F4">
+        <v>8.5306384024367493E-2</v>
+      </c>
+      <c r="G4">
+        <v>0.164726082735345</v>
+      </c>
+      <c r="H4">
+        <v>0.31961842353256698</v>
+      </c>
+      <c r="I4">
+        <v>2.7735243712533601E-2</v>
+      </c>
+      <c r="K4">
+        <v>6.4159740242030694E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="F6">
+        <v>-2.11324527447962E-2</v>
+      </c>
+      <c r="J6">
+        <v>-7.9580517746653201E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" ht="16" thickBot="1"/>
+    <row r="24" spans="2:14" ht="16" thickBot="1">
+      <c r="B24" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L24" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12">
-      <c r="A25" t="s">
-        <v>0</v>
-      </c>
-      <c r="B25" s="2">
-        <v>0.19377696556034199</v>
-      </c>
-      <c r="C25" s="2">
-        <v>0.14864047811018699</v>
-      </c>
-      <c r="D25" s="2">
-        <v>-3.4211729638660197E-2</v>
-      </c>
-      <c r="E25" s="2">
-        <v>7.7306317201005101E-2</v>
-      </c>
-      <c r="F25" s="2">
-        <v>7.4792693133144503E-2</v>
-      </c>
-      <c r="G25" s="2">
-        <v>4.4750492865178397E-2</v>
-      </c>
-      <c r="H25" s="2">
-        <v>7.0432480065617295E-2</v>
-      </c>
-      <c r="I25" s="2">
-        <v>0.36048404310182097</v>
-      </c>
-      <c r="J25" s="2">
-        <v>-3.5404714505740099E-2</v>
-      </c>
-      <c r="K25" s="2">
-        <v>-4.28184285195332E-2</v>
-      </c>
-      <c r="L25" s="2">
-        <v>-2.0043329745038099E-2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12">
-      <c r="A26" t="s">
-        <v>15</v>
-      </c>
-      <c r="B26" s="2">
-        <v>0.279459754945589</v>
+      <c r="C24" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+    </row>
+    <row r="25" spans="2:14">
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="5">
+        <v>0.15501406100000001</v>
+      </c>
+      <c r="D25" s="5">
+        <v>0.19431554300000001</v>
+      </c>
+      <c r="G25" s="5">
+        <v>0.34608744699999999</v>
+      </c>
+      <c r="H25" s="5">
+        <v>0.344955126</v>
+      </c>
+      <c r="I25" s="5">
+        <v>5.6733138000000002E-2</v>
+      </c>
+      <c r="J25" s="5">
+        <v>0.32515260699999998</v>
+      </c>
+      <c r="K25" s="5">
+        <v>0.36021372699999998</v>
+      </c>
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
+    </row>
+    <row r="26" spans="2:14">
+      <c r="B26" t="s">
+        <v>29</v>
       </c>
       <c r="C26" s="2">
-        <v>0.186479849778353</v>
+        <v>0.17621246643306199</v>
       </c>
       <c r="D26" s="2">
-        <v>-2.6943262605804801E-2</v>
-      </c>
-      <c r="E26" s="2">
-        <v>6.0648120765381001E-2</v>
-      </c>
-      <c r="F26" s="2">
-        <v>0.19411564298161599</v>
+        <v>0.24260531149436301</v>
       </c>
       <c r="G26" s="2">
-        <v>3.97435614897588E-2</v>
+        <v>0.39478523849170999</v>
       </c>
       <c r="H26" s="2">
-        <v>1.1062473397808701E-2</v>
+        <v>0.347969405722789</v>
       </c>
       <c r="I26" s="2">
-        <v>0.45083155711115303</v>
+        <v>6.2479996521071099E-2</v>
       </c>
       <c r="J26" s="2">
-        <v>-0.10923173784285101</v>
+        <v>0.35980824028866498</v>
       </c>
       <c r="K26" s="2">
-        <v>-2.61391764377291E-2</v>
-      </c>
-      <c r="L26" s="2">
-        <v>-1.971692084842E-2</v>
+        <v>0.44984631182524998</v>
+      </c>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
+    </row>
+    <row r="27" spans="2:14">
+      <c r="E27" s="5">
+        <v>-3.3343365999999999E-2</v>
+      </c>
+      <c r="F27" s="5">
+        <v>-4.9783518999999998E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14">
+      <c r="E28" s="2">
+        <v>-5.5149541840154297E-2</v>
+      </c>
+      <c r="F28" s="2">
+        <v>-5.6515245983640203E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>